<commit_message>
docs: finalize document review status
</commit_message>
<xml_diff>
--- a/doc/doc/新能源企业出海导航仪_D0数据标准冻结执行台账.xlsx
+++ b/doc/doc/新能源企业出海导航仪_D0数据标准冻结执行台账.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D0启动总览" sheetId="1" r:id="R756991b5b5d04511"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心实体冻结" sheetId="2" r:id="R04ab1ae1404c40fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心字段冻结" sheetId="3" r:id="R558b5f9525cd4eac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="枚举规则冻结" sheetId="4" r:id="R019b34c3f74a4936"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采集规范冻结" sheetId="5" r:id="R9ad75d4c4c7c40e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="质量规则冻结" sheetId="6" r:id="Rd1d08e0bb4634a92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首批国家范围" sheetId="7" r:id="R536a6bf62a4b46f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首批数据域目标" sheetId="8" r:id="R6be49f5a940a4ab0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D0任务计划" sheetId="9" r:id="R896a672aa4e44aa9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D0责任签署" sheetId="10" r:id="R1ebfff8437cc4622"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D0决策与变更" sheetId="11" r:id="R64a7b0305c3947e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D0验收签署" sheetId="12" r:id="Ra053542febe14472"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D0启动总览" sheetId="1" r:id="R487a6332bc2f43ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心实体冻结" sheetId="2" r:id="Rd6cbe2061e124980"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="核心字段冻结" sheetId="3" r:id="R58e4e778b76e4ee3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="枚举规则冻结" sheetId="4" r:id="R2860e1b1a8a74265"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="采集规范冻结" sheetId="5" r:id="R9592f189ccd441f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="质量规则冻结" sheetId="6" r:id="R1a26ab2d993b4250"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首批国家范围" sheetId="7" r:id="R7d83be6565bd40f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="首批数据域目标" sheetId="8" r:id="Rba5a0118eea84516"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D0任务计划" sheetId="9" r:id="R921db0776b454132"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D0责任签署" sheetId="10" r:id="R7164104ff4bc4f05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D0决策与变更" sheetId="11" r:id="R51816af00cb94a27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="D0验收签署" sheetId="12" r:id="R55bbf5386abb4bfd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,6 +24,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+  </x:numFmts>
   <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
@@ -110,7 +113,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="25">
+  <x:cellXfs count="28">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -158,6 +161,15 @@
     <x:xf numFmtId="0" fontId="4" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -169,7 +181,7 @@
         <x:color rgb="FF145C9E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF1F8"/>
         </x:patternFill>
       </x:fill>
@@ -180,7 +192,7 @@
         <x:color rgb="FF0F766E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD1FAE5"/>
         </x:patternFill>
       </x:fill>
@@ -191,7 +203,7 @@
         <x:color rgb="FF145C9E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF1F8"/>
         </x:patternFill>
       </x:fill>
@@ -202,7 +214,7 @@
         <x:color rgb="FF0F766E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD1FAE5"/>
         </x:patternFill>
       </x:fill>
@@ -213,7 +225,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE4E2"/>
         </x:patternFill>
       </x:fill>
@@ -224,7 +236,7 @@
         <x:color rgb="FF0F766E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD1FAE5"/>
         </x:patternFill>
       </x:fill>
@@ -235,7 +247,7 @@
         <x:color rgb="FF0F766E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD1FAE5"/>
         </x:patternFill>
       </x:fill>
@@ -246,7 +258,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE4E2"/>
         </x:patternFill>
       </x:fill>
@@ -257,7 +269,7 @@
         <x:color rgb="FFB54708"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF0C7"/>
         </x:patternFill>
       </x:fill>
@@ -298,8 +310,8 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="D0DecisionChangeTable" displayName="D0DecisionChangeTable" ref="A4:I7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:I7"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="D0DecisionChangeTable" displayName="D0DecisionChangeTable" ref="A4:I8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:I8"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="记录编号"/>
     <x:tableColumn id="2" name="类型"/>
@@ -706,7 +718,7 @@
     </x:row>
     <x:row r="2" ht="40" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>V1.0-BASELINE已发布；D0仅冻结数据标准与执行模板，不启动V0.1用户侧产品功能开发。</x:v>
+        <x:v>V1.0-BASELINE已于2026-07-30完成全部文档审核；D0仅冻结数据标准与执行模板，不启动V0.1用户侧产品功能开发。</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -759,7 +771,7 @@
         <x:v>正式成果可访问且版本一致</x:v>
       </x:c>
       <x:c r="F5" s="19" t="str">
-        <x:v>2026-07-24发布</x:v>
+        <x:v>2026-07-30完成全部文档审核；版本一致</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="43.20000076293945" hidden="0" customHeight="1">
@@ -918,7 +930,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09eb663c11f3452b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4383a6a064694d78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1140,7 +1152,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c55ac22e2644827"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde379747267e4f83"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1307,6 +1319,35 @@
       </x:c>
       <x:c r="I7" s="19" t="str"/>
     </x:row>
+    <x:row r="8" ht="64.80000305175781" customHeight="1">
+      <x:c r="A8" s="26" t="str">
+        <x:v>D0-DEC-004</x:v>
+      </x:c>
+      <x:c r="B8" s="26" t="str">
+        <x:v>决定</x:v>
+      </x:c>
+      <x:c r="C8" s="26" t="str">
+        <x:v>全部文档审核完成</x:v>
+      </x:c>
+      <x:c r="D8" s="26" t="str">
+        <x:v>Word总文档、Markdown分册、Excel技术附件、首批数据采集实施方案及D0执行台账完成审核并纳入V1.0-BASELINE</x:v>
+      </x:c>
+      <x:c r="E8" s="26" t="str">
+        <x:v>用户确认所有文档审核完成；执行类状态仍以实际证据更新</x:v>
+      </x:c>
+      <x:c r="F8" s="26" t="str">
+        <x:v>项目编制组</x:v>
+      </x:c>
+      <x:c r="G8" s="26" t="str">
+        <x:v>用户确认</x:v>
+      </x:c>
+      <x:c r="H8" s="26" t="str">
+        <x:v>已生效</x:v>
+      </x:c>
+      <x:c r="I8" s="27" t="n">
+        <x:v>46233</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:I1"/>
@@ -1322,7 +1363,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbce471bf39fc48ba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2565e8110ceb407a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1598,7 +1639,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R895e79b4f279402d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb7a4a22548e4243"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2498,7 +2539,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd02edbca41cd4625"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra08a5ca038c748be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6108,7 +6149,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb5198f5245d4c0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa70947b5193469a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12730,7 +12771,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfdd72747df974dfa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c3eee36e1204b41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12775,7 +12816,7 @@
     </x:row>
     <x:row r="2" ht="40" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>采集频率与业务复核周期分开；自动任务先写L0和运行日志，再进入暂存、质量、审核和发布链。</x:v>
+        <x:v>规则文档已确认；采集频率与业务复核周期分开，实际生效仍须完成D0冻结及责任签署。</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -12892,7 +12933,7 @@
         <x:v>FR-COLLECT-001;006;007</x:v>
       </x:c>
       <x:c r="N5" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -12936,7 +12977,7 @@
         <x:v>FR-COLLECT-003;005;006</x:v>
       </x:c>
       <x:c r="N6" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -12980,7 +13021,7 @@
         <x:v>FR-COLLECT-002;003;005</x:v>
       </x:c>
       <x:c r="N7" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -13024,7 +13065,7 @@
         <x:v>FR-COLLECT-002;003;005;007</x:v>
       </x:c>
       <x:c r="N8" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -13068,7 +13109,7 @@
         <x:v>FR-COLLECT-003;005;006</x:v>
       </x:c>
       <x:c r="N9" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -13112,7 +13153,7 @@
         <x:v>FR-COLLECT-002;003;005</x:v>
       </x:c>
       <x:c r="N10" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -13156,7 +13197,7 @@
         <x:v>FR-COLLECT-005;007</x:v>
       </x:c>
       <x:c r="N11" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -13200,7 +13241,7 @@
         <x:v>FR-COLLECT-003;006</x:v>
       </x:c>
       <x:c r="N12" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="43.20000076293945" hidden="0" customHeight="1">
@@ -13244,7 +13285,7 @@
         <x:v>FR-COLLECT-003;006;007</x:v>
       </x:c>
       <x:c r="N13" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="43.20000076293945" hidden="0" customHeight="1">
@@ -13288,7 +13329,7 @@
         <x:v>FR-COLLECT-004;007</x:v>
       </x:c>
       <x:c r="N14" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="43.20000076293945" hidden="0" customHeight="1">
@@ -13332,7 +13373,7 @@
         <x:v>FR-COLLECT-004;007</x:v>
       </x:c>
       <x:c r="N15" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="43.20000076293945" hidden="0" customHeight="1">
@@ -13376,7 +13417,7 @@
         <x:v>FR-COLLECT-006</x:v>
       </x:c>
       <x:c r="N16" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -13420,7 +13461,7 @@
         <x:v>FR-DATA-006;FR-COLLECT-001;007</x:v>
       </x:c>
       <x:c r="N17" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -13464,7 +13505,7 @@
         <x:v>FR-COLLECT-003;006</x:v>
       </x:c>
       <x:c r="N18" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -13474,7 +13515,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbd432d6500384efc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R939b47378f07444d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13517,7 +13558,7 @@
     </x:row>
     <x:row r="2" ht="40" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>质量状态只使用passed/warning/failed/conflicted；时效、权限和发布状态独立。P0问题不能被平均分抵消，豁免必须到期。</x:v>
+        <x:v>规则文档已确认；质量状态、发布门禁和豁免约束实际生效仍须完成D0冻结及验收。</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -13623,7 +13664,7 @@
         <x:v>FR-COLLECT-001;007</x:v>
       </x:c>
       <x:c r="L5" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M5" s="19" t="str">
         <x:v>公开可访问不等于可再分发</x:v>
@@ -13664,7 +13705,7 @@
         <x:v>FR-COLLECT-002;FR-QUALITY-005</x:v>
       </x:c>
       <x:c r="L6" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M6" s="24" t="str">
         <x:v>链路完整率要求100%</x:v>
@@ -13705,7 +13746,7 @@
         <x:v>FR-QUALITY-001</x:v>
       </x:c>
       <x:c r="L7" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M7" s="19" t="str">
         <x:v>依法删除走受控任务</x:v>
@@ -13746,7 +13787,7 @@
         <x:v>FR-QUALITY-002</x:v>
       </x:c>
       <x:c r="L8" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M8" s="24" t="str">
         <x:v>not_applicable须有依据</x:v>
@@ -13787,7 +13828,7 @@
         <x:v>FR-QUALITY-003</x:v>
       </x:c>
       <x:c r="L9" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M9" s="19" t="str">
         <x:v>保留历史ID映射</x:v>
@@ -13828,7 +13869,7 @@
         <x:v>FR-QUALITY-004</x:v>
       </x:c>
       <x:c r="L10" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M10" s="24" t="str">
         <x:v>过程态另用工作流</x:v>
@@ -13869,7 +13910,7 @@
         <x:v>FR-QUALITY-007</x:v>
       </x:c>
       <x:c r="L11" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M11" s="19" t="str">
         <x:v>quality_status保持独立</x:v>
@@ -13910,7 +13951,7 @@
         <x:v>FR-QUALITY-005;006</x:v>
       </x:c>
       <x:c r="L12" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M12" s="24" t="str">
         <x:v>不使用多数票自动覆盖</x:v>
@@ -13951,7 +13992,7 @@
         <x:v>FR-QUALITY-006</x:v>
       </x:c>
       <x:c r="L13" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M13" s="19" t="str">
         <x:v>历史版本不可覆盖</x:v>
@@ -13992,7 +14033,7 @@
         <x:v>FR-DATA-006;FR-QUALITY-007</x:v>
       </x:c>
       <x:c r="L14" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M14" s="24" t="str">
         <x:v>权限先于索引检索</x:v>
@@ -14033,7 +14074,7 @@
         <x:v>FR-SCORE-001</x:v>
       </x:c>
       <x:c r="L15" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M15" s="19" t="str">
         <x:v>low/medium/high/critical</x:v>
@@ -14074,7 +14115,7 @@
         <x:v>FR-QUALITY-006;FR-SCORE-001</x:v>
       </x:c>
       <x:c r="L16" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M16" s="24" t="str">
         <x:v>疑似虚假为独立标记</x:v>
@@ -14115,7 +14156,7 @@
         <x:v>FR-SCORE-001</x:v>
       </x:c>
       <x:c r="L17" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M17" s="19" t="str">
         <x:v>同模型变体分别校验</x:v>
@@ -14156,7 +14197,7 @@
         <x:v>FR-DATA-005;FR-QUALITY-005</x:v>
       </x:c>
       <x:c r="L18" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M18" s="24" t="str">
         <x:v>印尼另过专项验收</x:v>
@@ -14197,7 +14238,7 @@
         <x:v>FR-QUALITY-008</x:v>
       </x:c>
       <x:c r="L19" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M19" s="19" t="str">
         <x:v>P0豁免不改变原严重度</x:v>
@@ -14238,7 +14279,7 @@
         <x:v>FR-QUALITY-008</x:v>
       </x:c>
       <x:c r="L20" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>文档已确认；待D0冻结</x:v>
       </x:c>
       <x:c r="M20" s="24" t="str">
         <x:v>P0单独计数且不可被平均</x:v>
@@ -14251,7 +14292,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R002d676dd7664d5a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89a2bd9cdfcd43a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14363,7 +14404,7 @@
         <x:v>不可无批准替换</x:v>
       </x:c>
       <x:c r="I5" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>范围已确认</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -14392,7 +14433,7 @@
         <x:v>来源/语言风险可走变更</x:v>
       </x:c>
       <x:c r="I6" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>范围已确认</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -14421,7 +14462,7 @@
         <x:v>来源/语言风险可走变更</x:v>
       </x:c>
       <x:c r="I7" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>范围已确认</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -14450,7 +14491,7 @@
         <x:v>来源风险可走变更</x:v>
       </x:c>
       <x:c r="I8" s="24" t="str">
-        <x:v>候选</x:v>
+        <x:v>范围已确认</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -14479,7 +14520,7 @@
         <x:v>来源/语言风险可走变更</x:v>
       </x:c>
       <x:c r="I9" s="19" t="str">
-        <x:v>候选</x:v>
+        <x:v>范围已确认</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14489,7 +14530,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2547f51deebf4a54"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5014d76831cc4776"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14775,7 +14816,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44a6d68475e74779"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6fb48f7bdf7c4c75"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15041,7 +15082,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbff4b310be4c4e71"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bb85e3b589b41ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>